<commit_message>
data(m10): nap so booking T9 (45 lead tiec, DT chot 140,9 tr) + chi phi ads NEC T9 tu API M5.1
- scripts/build-booking-ads.mjs: keo chien dich funnel=booking tu Postgres M5.1 cho thang chua co file Meta Ads
- build-data.mjs: gop booking_ads_api.json (chi them; thang co file Meta Ads thi file thang)
- hub.ts: them truong tuy chon booking_meta.ads_api_months; BookingView khong bao thieu bao cao ads cho thang nay
- docs/modules/M10_Booking.md: muc 6b so T9

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_input/monthly/2025-10.xlsx
+++ b/data_input/monthly/2025-10.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,12 +35,8 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00F3F2EE"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -57,11 +53,6 @@
         <fgColor rgb="FFF2EFE6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F1F26"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -75,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -87,7 +78,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -943,29 +933,36 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>used</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>rev</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>disc</t>
         </is>

</xml_diff>